<commit_message>
Add recipient email addresses to the shared application ledger
</commit_message>
<xml_diff>
--- a/heymail/assets/templates/application-ledger.xlsx
+++ b/heymail/assets/templates/application-ledger.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="投递台账" sheetId="1" r:id="R0f33f66f19cd4f1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="投递台账" sheetId="1" r:id="R42573c6d52bc4dda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -358,13 +358,13 @@
     <xdr:ext cx="2571750" cy="663963"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="19b34e3b-1001-45de-950c-8bca265d4786"/>
+        <xdr:cNvPr id="1" name="523470c7-47ce-47dc-8d8e-f5be2200c4c7"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf20a89d276d84dcb"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9e23238569b6422f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -377,7 +377,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>952500</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
@@ -385,13 +385,13 @@
     <xdr:ext cx="2667000" cy="323620"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="6831f407-6e9d-45bf-9808-f56181ee17de"/>
+        <xdr:cNvPr id="2" name="d9ff7376-ccf8-4d53-b1bf-fa7092390344"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R40175a8a6a284f23"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R841af973b41c4958"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -406,18 +406,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ApplicationsTable" displayName="ApplicationsTable" ref="A4:I24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:I24"/>
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ApplicationsTable" displayName="ApplicationsTable" ref="A4:J24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:J24"/>
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="公司"/>
     <x:tableColumn id="2" name="岗位"/>
     <x:tableColumn id="3" name="工作地点"/>
     <x:tableColumn id="4" name="投递时间"/>
     <x:tableColumn id="5" name="投递 Agent"/>
-    <x:tableColumn id="6" name="当前进展"/>
-    <x:tableColumn id="7" name="下次跟进"/>
-    <x:tableColumn id="8" name="备注"/>
-    <x:tableColumn id="9" name="_record_id"/>
+    <x:tableColumn id="6" name="收件邮箱"/>
+    <x:tableColumn id="7" name="当前进展"/>
+    <x:tableColumn id="8" name="下次跟进"/>
+    <x:tableColumn id="9" name="备注"/>
+    <x:tableColumn id="10" name="_record_id"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -626,10 +627,11 @@
     <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="43" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="14" hidden="1" customWidth="1"/>
+    <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="43" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="8" customHeight="1">
@@ -641,6 +643,7 @@
       <x:c r="F1" s="1"/>
       <x:c r="G1" s="1"/>
       <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="1"/>
@@ -653,6 +656,7 @@
       <x:c r="F2" s="1"/>
       <x:c r="G2" s="1"/>
       <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="4"/>
@@ -663,6 +667,7 @@
       <x:c r="F3" s="4"/>
       <x:c r="G3" s="4"/>
       <x:c r="H3" s="4"/>
+      <x:c r="I3" s="4"/>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -681,15 +686,18 @@
         <x:v>投递 Agent</x:v>
       </x:c>
       <x:c r="F4" s="11" t="str">
+        <x:v>收件邮箱</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="str">
         <x:v>当前进展</x:v>
       </x:c>
-      <x:c r="G4" s="11" t="str">
+      <x:c r="H4" s="11" t="str">
         <x:v>下次跟进</x:v>
       </x:c>
-      <x:c r="H4" s="11" t="str">
+      <x:c r="I4" s="11" t="str">
         <x:v>备注</x:v>
       </x:c>
-      <x:c r="I4" s="11" t="str">
+      <x:c r="J4" s="11" t="str">
         <x:v>_record_id</x:v>
       </x:c>
     </x:row>
@@ -699,10 +707,11 @@
       <x:c r="C5" s="32"/>
       <x:c r="D5" s="33"/>
       <x:c r="E5" s="34"/>
-      <x:c r="F5" s="39"/>
-      <x:c r="G5" s="40"/>
-      <x:c r="H5" s="41"/>
-      <x:c r="I5" s="38"/>
+      <x:c r="F5" s="31"/>
+      <x:c r="G5" s="39"/>
+      <x:c r="H5" s="40"/>
+      <x:c r="I5" s="41"/>
+      <x:c r="J5" s="38"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="50"/>
@@ -710,10 +719,11 @@
       <x:c r="C6" s="51"/>
       <x:c r="D6" s="52"/>
       <x:c r="E6" s="53"/>
-      <x:c r="F6" s="39"/>
-      <x:c r="G6" s="40"/>
-      <x:c r="H6" s="58"/>
-      <x:c r="I6" s="57"/>
+      <x:c r="F6" s="50"/>
+      <x:c r="G6" s="39"/>
+      <x:c r="H6" s="40"/>
+      <x:c r="I6" s="58"/>
+      <x:c r="J6" s="57"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="31"/>
@@ -721,10 +731,11 @@
       <x:c r="C7" s="32"/>
       <x:c r="D7" s="33"/>
       <x:c r="E7" s="34"/>
-      <x:c r="F7" s="39"/>
-      <x:c r="G7" s="40"/>
-      <x:c r="H7" s="41"/>
-      <x:c r="I7" s="38"/>
+      <x:c r="F7" s="31"/>
+      <x:c r="G7" s="39"/>
+      <x:c r="H7" s="40"/>
+      <x:c r="I7" s="41"/>
+      <x:c r="J7" s="38"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="50"/>
@@ -732,10 +743,11 @@
       <x:c r="C8" s="51"/>
       <x:c r="D8" s="52"/>
       <x:c r="E8" s="53"/>
-      <x:c r="F8" s="39"/>
-      <x:c r="G8" s="40"/>
-      <x:c r="H8" s="58"/>
-      <x:c r="I8" s="57"/>
+      <x:c r="F8" s="50"/>
+      <x:c r="G8" s="39"/>
+      <x:c r="H8" s="40"/>
+      <x:c r="I8" s="58"/>
+      <x:c r="J8" s="57"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="31"/>
@@ -743,10 +755,11 @@
       <x:c r="C9" s="32"/>
       <x:c r="D9" s="33"/>
       <x:c r="E9" s="34"/>
-      <x:c r="F9" s="39"/>
-      <x:c r="G9" s="40"/>
-      <x:c r="H9" s="41"/>
-      <x:c r="I9" s="38"/>
+      <x:c r="F9" s="31"/>
+      <x:c r="G9" s="39"/>
+      <x:c r="H9" s="40"/>
+      <x:c r="I9" s="41"/>
+      <x:c r="J9" s="38"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="50"/>
@@ -754,10 +767,11 @@
       <x:c r="C10" s="51"/>
       <x:c r="D10" s="52"/>
       <x:c r="E10" s="53"/>
-      <x:c r="F10" s="39"/>
-      <x:c r="G10" s="40"/>
-      <x:c r="H10" s="58"/>
-      <x:c r="I10" s="57"/>
+      <x:c r="F10" s="50"/>
+      <x:c r="G10" s="39"/>
+      <x:c r="H10" s="40"/>
+      <x:c r="I10" s="58"/>
+      <x:c r="J10" s="57"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="31"/>
@@ -765,10 +779,11 @@
       <x:c r="C11" s="32"/>
       <x:c r="D11" s="33"/>
       <x:c r="E11" s="34"/>
-      <x:c r="F11" s="39"/>
-      <x:c r="G11" s="40"/>
-      <x:c r="H11" s="41"/>
-      <x:c r="I11" s="38"/>
+      <x:c r="F11" s="31"/>
+      <x:c r="G11" s="39"/>
+      <x:c r="H11" s="40"/>
+      <x:c r="I11" s="41"/>
+      <x:c r="J11" s="38"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="50"/>
@@ -776,10 +791,11 @@
       <x:c r="C12" s="51"/>
       <x:c r="D12" s="52"/>
       <x:c r="E12" s="53"/>
-      <x:c r="F12" s="39"/>
-      <x:c r="G12" s="40"/>
-      <x:c r="H12" s="58"/>
-      <x:c r="I12" s="57"/>
+      <x:c r="F12" s="50"/>
+      <x:c r="G12" s="39"/>
+      <x:c r="H12" s="40"/>
+      <x:c r="I12" s="58"/>
+      <x:c r="J12" s="57"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="31"/>
@@ -787,10 +803,11 @@
       <x:c r="C13" s="32"/>
       <x:c r="D13" s="33"/>
       <x:c r="E13" s="34"/>
-      <x:c r="F13" s="39"/>
-      <x:c r="G13" s="40"/>
-      <x:c r="H13" s="41"/>
-      <x:c r="I13" s="38"/>
+      <x:c r="F13" s="31"/>
+      <x:c r="G13" s="39"/>
+      <x:c r="H13" s="40"/>
+      <x:c r="I13" s="41"/>
+      <x:c r="J13" s="38"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="50"/>
@@ -798,10 +815,11 @@
       <x:c r="C14" s="51"/>
       <x:c r="D14" s="52"/>
       <x:c r="E14" s="53"/>
-      <x:c r="F14" s="39"/>
-      <x:c r="G14" s="40"/>
-      <x:c r="H14" s="58"/>
-      <x:c r="I14" s="57"/>
+      <x:c r="F14" s="50"/>
+      <x:c r="G14" s="39"/>
+      <x:c r="H14" s="40"/>
+      <x:c r="I14" s="58"/>
+      <x:c r="J14" s="57"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="31"/>
@@ -809,10 +827,11 @@
       <x:c r="C15" s="32"/>
       <x:c r="D15" s="33"/>
       <x:c r="E15" s="34"/>
-      <x:c r="F15" s="39"/>
-      <x:c r="G15" s="40"/>
-      <x:c r="H15" s="41"/>
-      <x:c r="I15" s="38"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="39"/>
+      <x:c r="H15" s="40"/>
+      <x:c r="I15" s="41"/>
+      <x:c r="J15" s="38"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="50"/>
@@ -820,10 +839,11 @@
       <x:c r="C16" s="51"/>
       <x:c r="D16" s="52"/>
       <x:c r="E16" s="53"/>
-      <x:c r="F16" s="39"/>
-      <x:c r="G16" s="40"/>
-      <x:c r="H16" s="58"/>
-      <x:c r="I16" s="57"/>
+      <x:c r="F16" s="50"/>
+      <x:c r="G16" s="39"/>
+      <x:c r="H16" s="40"/>
+      <x:c r="I16" s="58"/>
+      <x:c r="J16" s="57"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="31"/>
@@ -831,10 +851,11 @@
       <x:c r="C17" s="32"/>
       <x:c r="D17" s="33"/>
       <x:c r="E17" s="34"/>
-      <x:c r="F17" s="39"/>
-      <x:c r="G17" s="40"/>
-      <x:c r="H17" s="41"/>
-      <x:c r="I17" s="38"/>
+      <x:c r="F17" s="31"/>
+      <x:c r="G17" s="39"/>
+      <x:c r="H17" s="40"/>
+      <x:c r="I17" s="41"/>
+      <x:c r="J17" s="38"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="50"/>
@@ -842,10 +863,11 @@
       <x:c r="C18" s="51"/>
       <x:c r="D18" s="52"/>
       <x:c r="E18" s="53"/>
-      <x:c r="F18" s="39"/>
-      <x:c r="G18" s="40"/>
-      <x:c r="H18" s="58"/>
-      <x:c r="I18" s="57"/>
+      <x:c r="F18" s="50"/>
+      <x:c r="G18" s="39"/>
+      <x:c r="H18" s="40"/>
+      <x:c r="I18" s="58"/>
+      <x:c r="J18" s="57"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="31"/>
@@ -853,10 +875,11 @@
       <x:c r="C19" s="32"/>
       <x:c r="D19" s="33"/>
       <x:c r="E19" s="34"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="40"/>
-      <x:c r="H19" s="41"/>
-      <x:c r="I19" s="38"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="40"/>
+      <x:c r="I19" s="41"/>
+      <x:c r="J19" s="38"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="50"/>
@@ -864,10 +887,11 @@
       <x:c r="C20" s="51"/>
       <x:c r="D20" s="52"/>
       <x:c r="E20" s="53"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="40"/>
-      <x:c r="H20" s="58"/>
-      <x:c r="I20" s="57"/>
+      <x:c r="F20" s="50"/>
+      <x:c r="G20" s="39"/>
+      <x:c r="H20" s="40"/>
+      <x:c r="I20" s="58"/>
+      <x:c r="J20" s="57"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="31"/>
@@ -875,10 +899,11 @@
       <x:c r="C21" s="32"/>
       <x:c r="D21" s="33"/>
       <x:c r="E21" s="34"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="40"/>
-      <x:c r="H21" s="41"/>
-      <x:c r="I21" s="38"/>
+      <x:c r="F21" s="31"/>
+      <x:c r="G21" s="39"/>
+      <x:c r="H21" s="40"/>
+      <x:c r="I21" s="41"/>
+      <x:c r="J21" s="38"/>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="50"/>
@@ -886,10 +911,11 @@
       <x:c r="C22" s="51"/>
       <x:c r="D22" s="52"/>
       <x:c r="E22" s="53"/>
-      <x:c r="F22" s="39"/>
-      <x:c r="G22" s="40"/>
-      <x:c r="H22" s="58"/>
-      <x:c r="I22" s="57"/>
+      <x:c r="F22" s="50"/>
+      <x:c r="G22" s="39"/>
+      <x:c r="H22" s="40"/>
+      <x:c r="I22" s="58"/>
+      <x:c r="J22" s="57"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="31"/>
@@ -897,10 +923,11 @@
       <x:c r="C23" s="32"/>
       <x:c r="D23" s="33"/>
       <x:c r="E23" s="34"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="40"/>
-      <x:c r="H23" s="41"/>
-      <x:c r="I23" s="38"/>
+      <x:c r="F23" s="31"/>
+      <x:c r="G23" s="39"/>
+      <x:c r="H23" s="40"/>
+      <x:c r="I23" s="41"/>
+      <x:c r="J23" s="38"/>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="50"/>
@@ -908,13 +935,14 @@
       <x:c r="C24" s="51"/>
       <x:c r="D24" s="52"/>
       <x:c r="E24" s="53"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="40"/>
-      <x:c r="H24" s="58"/>
-      <x:c r="I24" s="57"/>
+      <x:c r="F24" s="50"/>
+      <x:c r="G24" s="39"/>
+      <x:c r="H24" s="40"/>
+      <x:c r="I24" s="58"/>
+      <x:c r="J24" s="57"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F5:F200">
+  <x:conditionalFormatting sqref="G5:G200">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <x:formula>"已投递"</x:formula>
     </x:cfRule>
@@ -934,20 +962,20 @@
       <x:formula>"已放弃"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G5:G200">
+  <x:conditionalFormatting sqref="H5:H200">
     <x:cfRule type="expression" dxfId="6" priority="7">
-      <x:formula>AND(ISNUMBER(G5),G5&lt;=TODAY(),$F5&lt;&gt;"已录用",$F5&lt;&gt;"未通过",$F5&lt;&gt;"已放弃")</x:formula>
+      <x:formula>AND(ISNUMBER(H5),H5&lt;=TODAY(),$G5&lt;&gt;"已录用",$G5&lt;&gt;"未通过",$G5&lt;&gt;"已放弃")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="F5:F200">
+    <x:dataValidation type="list" sqref="G5:G200">
       <x:formula1>"已投递,已回复,面试中,已录用,未通过,已放弃,投递失败,发送待核实"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdffe6bb65ea4feb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63612bb17a4848a1"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd59447653e7a478e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R682da7e077b249bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Replace next follow-up date with latest progress notes
</commit_message>
<xml_diff>
--- a/heymail/assets/templates/application-ledger.xlsx
+++ b/heymail/assets/templates/application-ledger.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="投递台账" sheetId="1" r:id="R42573c6d52bc4dda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="投递台账" sheetId="1" r:id="Rffd3d8ac3f694e28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd hh:mm"/>
-    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="201" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -118,7 +118,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -158,14 +158,17 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -192,7 +195,7 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -216,7 +219,7 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -228,7 +231,7 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -249,7 +252,7 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -273,7 +276,7 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="3" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -288,7 +291,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="6">
     <x:dxf>
       <x:fill>
         <x:patternFill patternType="solid">
@@ -331,17 +334,6 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9B2C20"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFBE0D9"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -358,13 +350,13 @@
     <xdr:ext cx="2571750" cy="663963"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="523470c7-47ce-47dc-8d8e-f5be2200c4c7"/>
+        <xdr:cNvPr id="1" name="6d63a8bb-5429-4a17-a341-f3a9b2348153"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9e23238569b6422f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3360a65194004531"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -385,13 +377,13 @@
     <xdr:ext cx="2667000" cy="323620"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="d9ff7376-ccf8-4d53-b1bf-fa7092390344"/>
+        <xdr:cNvPr id="2" name="11d53529-7c6c-4b8e-8c2f-7da8315c758f"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R841af973b41c4958"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R43ae6279d98d4003"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -416,7 +408,7 @@
     <x:tableColumn id="5" name="投递 Agent"/>
     <x:tableColumn id="6" name="收件邮箱"/>
     <x:tableColumn id="7" name="当前进展"/>
-    <x:tableColumn id="8" name="下次跟进"/>
+    <x:tableColumn id="8" name="最新进展"/>
     <x:tableColumn id="9" name="备注"/>
     <x:tableColumn id="10" name="_record_id"/>
   </x:tableColumns>
@@ -629,7 +621,7 @@
     <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="43" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="14" hidden="1" customWidth="1"/>
   </x:cols>
@@ -692,7 +684,7 @@
         <x:v>当前进展</x:v>
       </x:c>
       <x:c r="H4" s="11" t="str">
-        <x:v>下次跟进</x:v>
+        <x:v>最新进展</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
         <x:v>备注</x:v>
@@ -702,244 +694,244 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
-      <x:c r="A5" s="31"/>
-      <x:c r="B5" s="31"/>
-      <x:c r="C5" s="32"/>
-      <x:c r="D5" s="33"/>
-      <x:c r="E5" s="34"/>
-      <x:c r="F5" s="31"/>
-      <x:c r="G5" s="39"/>
-      <x:c r="H5" s="40"/>
-      <x:c r="I5" s="41"/>
-      <x:c r="J5" s="38"/>
+      <x:c r="A5" s="32"/>
+      <x:c r="B5" s="32"/>
+      <x:c r="C5" s="33"/>
+      <x:c r="D5" s="34"/>
+      <x:c r="E5" s="35"/>
+      <x:c r="F5" s="32"/>
+      <x:c r="G5" s="40"/>
+      <x:c r="H5" s="41"/>
+      <x:c r="I5" s="42"/>
+      <x:c r="J5" s="39"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
-      <x:c r="A6" s="50"/>
-      <x:c r="B6" s="50"/>
-      <x:c r="C6" s="51"/>
-      <x:c r="D6" s="52"/>
-      <x:c r="E6" s="53"/>
-      <x:c r="F6" s="50"/>
-      <x:c r="G6" s="39"/>
-      <x:c r="H6" s="40"/>
-      <x:c r="I6" s="58"/>
-      <x:c r="J6" s="57"/>
+      <x:c r="A6" s="51"/>
+      <x:c r="B6" s="51"/>
+      <x:c r="C6" s="52"/>
+      <x:c r="D6" s="53"/>
+      <x:c r="E6" s="54"/>
+      <x:c r="F6" s="51"/>
+      <x:c r="G6" s="40"/>
+      <x:c r="H6" s="41"/>
+      <x:c r="I6" s="59"/>
+      <x:c r="J6" s="58"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
-      <x:c r="A7" s="31"/>
-      <x:c r="B7" s="31"/>
-      <x:c r="C7" s="32"/>
-      <x:c r="D7" s="33"/>
-      <x:c r="E7" s="34"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="39"/>
-      <x:c r="H7" s="40"/>
-      <x:c r="I7" s="41"/>
-      <x:c r="J7" s="38"/>
+      <x:c r="A7" s="32"/>
+      <x:c r="B7" s="32"/>
+      <x:c r="C7" s="33"/>
+      <x:c r="D7" s="34"/>
+      <x:c r="E7" s="35"/>
+      <x:c r="F7" s="32"/>
+      <x:c r="G7" s="40"/>
+      <x:c r="H7" s="41"/>
+      <x:c r="I7" s="42"/>
+      <x:c r="J7" s="39"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
-      <x:c r="A8" s="50"/>
-      <x:c r="B8" s="50"/>
-      <x:c r="C8" s="51"/>
-      <x:c r="D8" s="52"/>
-      <x:c r="E8" s="53"/>
-      <x:c r="F8" s="50"/>
-      <x:c r="G8" s="39"/>
-      <x:c r="H8" s="40"/>
-      <x:c r="I8" s="58"/>
-      <x:c r="J8" s="57"/>
+      <x:c r="A8" s="51"/>
+      <x:c r="B8" s="51"/>
+      <x:c r="C8" s="52"/>
+      <x:c r="D8" s="53"/>
+      <x:c r="E8" s="54"/>
+      <x:c r="F8" s="51"/>
+      <x:c r="G8" s="40"/>
+      <x:c r="H8" s="41"/>
+      <x:c r="I8" s="59"/>
+      <x:c r="J8" s="58"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
-      <x:c r="A9" s="31"/>
-      <x:c r="B9" s="31"/>
-      <x:c r="C9" s="32"/>
-      <x:c r="D9" s="33"/>
-      <x:c r="E9" s="34"/>
-      <x:c r="F9" s="31"/>
-      <x:c r="G9" s="39"/>
-      <x:c r="H9" s="40"/>
-      <x:c r="I9" s="41"/>
-      <x:c r="J9" s="38"/>
+      <x:c r="A9" s="32"/>
+      <x:c r="B9" s="32"/>
+      <x:c r="C9" s="33"/>
+      <x:c r="D9" s="34"/>
+      <x:c r="E9" s="35"/>
+      <x:c r="F9" s="32"/>
+      <x:c r="G9" s="40"/>
+      <x:c r="H9" s="41"/>
+      <x:c r="I9" s="42"/>
+      <x:c r="J9" s="39"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
-      <x:c r="A10" s="50"/>
-      <x:c r="B10" s="50"/>
-      <x:c r="C10" s="51"/>
-      <x:c r="D10" s="52"/>
-      <x:c r="E10" s="53"/>
-      <x:c r="F10" s="50"/>
-      <x:c r="G10" s="39"/>
-      <x:c r="H10" s="40"/>
-      <x:c r="I10" s="58"/>
-      <x:c r="J10" s="57"/>
+      <x:c r="A10" s="51"/>
+      <x:c r="B10" s="51"/>
+      <x:c r="C10" s="52"/>
+      <x:c r="D10" s="53"/>
+      <x:c r="E10" s="54"/>
+      <x:c r="F10" s="51"/>
+      <x:c r="G10" s="40"/>
+      <x:c r="H10" s="41"/>
+      <x:c r="I10" s="59"/>
+      <x:c r="J10" s="58"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="31"/>
-      <x:c r="B11" s="31"/>
-      <x:c r="C11" s="32"/>
-      <x:c r="D11" s="33"/>
-      <x:c r="E11" s="34"/>
-      <x:c r="F11" s="31"/>
-      <x:c r="G11" s="39"/>
-      <x:c r="H11" s="40"/>
-      <x:c r="I11" s="41"/>
-      <x:c r="J11" s="38"/>
+      <x:c r="A11" s="32"/>
+      <x:c r="B11" s="32"/>
+      <x:c r="C11" s="33"/>
+      <x:c r="D11" s="34"/>
+      <x:c r="E11" s="35"/>
+      <x:c r="F11" s="32"/>
+      <x:c r="G11" s="40"/>
+      <x:c r="H11" s="41"/>
+      <x:c r="I11" s="42"/>
+      <x:c r="J11" s="39"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="50"/>
-      <x:c r="B12" s="50"/>
-      <x:c r="C12" s="51"/>
-      <x:c r="D12" s="52"/>
-      <x:c r="E12" s="53"/>
-      <x:c r="F12" s="50"/>
-      <x:c r="G12" s="39"/>
-      <x:c r="H12" s="40"/>
-      <x:c r="I12" s="58"/>
-      <x:c r="J12" s="57"/>
+      <x:c r="A12" s="51"/>
+      <x:c r="B12" s="51"/>
+      <x:c r="C12" s="52"/>
+      <x:c r="D12" s="53"/>
+      <x:c r="E12" s="54"/>
+      <x:c r="F12" s="51"/>
+      <x:c r="G12" s="40"/>
+      <x:c r="H12" s="41"/>
+      <x:c r="I12" s="59"/>
+      <x:c r="J12" s="58"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="31"/>
-      <x:c r="B13" s="31"/>
-      <x:c r="C13" s="32"/>
-      <x:c r="D13" s="33"/>
-      <x:c r="E13" s="34"/>
-      <x:c r="F13" s="31"/>
-      <x:c r="G13" s="39"/>
-      <x:c r="H13" s="40"/>
-      <x:c r="I13" s="41"/>
-      <x:c r="J13" s="38"/>
+      <x:c r="A13" s="32"/>
+      <x:c r="B13" s="32"/>
+      <x:c r="C13" s="33"/>
+      <x:c r="D13" s="34"/>
+      <x:c r="E13" s="35"/>
+      <x:c r="F13" s="32"/>
+      <x:c r="G13" s="40"/>
+      <x:c r="H13" s="41"/>
+      <x:c r="I13" s="42"/>
+      <x:c r="J13" s="39"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="50"/>
-      <x:c r="B14" s="50"/>
-      <x:c r="C14" s="51"/>
-      <x:c r="D14" s="52"/>
-      <x:c r="E14" s="53"/>
-      <x:c r="F14" s="50"/>
-      <x:c r="G14" s="39"/>
-      <x:c r="H14" s="40"/>
-      <x:c r="I14" s="58"/>
-      <x:c r="J14" s="57"/>
+      <x:c r="A14" s="51"/>
+      <x:c r="B14" s="51"/>
+      <x:c r="C14" s="52"/>
+      <x:c r="D14" s="53"/>
+      <x:c r="E14" s="54"/>
+      <x:c r="F14" s="51"/>
+      <x:c r="G14" s="40"/>
+      <x:c r="H14" s="41"/>
+      <x:c r="I14" s="59"/>
+      <x:c r="J14" s="58"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="31"/>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="32"/>
-      <x:c r="D15" s="33"/>
-      <x:c r="E15" s="34"/>
-      <x:c r="F15" s="31"/>
-      <x:c r="G15" s="39"/>
-      <x:c r="H15" s="40"/>
-      <x:c r="I15" s="41"/>
-      <x:c r="J15" s="38"/>
+      <x:c r="A15" s="32"/>
+      <x:c r="B15" s="32"/>
+      <x:c r="C15" s="33"/>
+      <x:c r="D15" s="34"/>
+      <x:c r="E15" s="35"/>
+      <x:c r="F15" s="32"/>
+      <x:c r="G15" s="40"/>
+      <x:c r="H15" s="41"/>
+      <x:c r="I15" s="42"/>
+      <x:c r="J15" s="39"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
-      <x:c r="A16" s="50"/>
-      <x:c r="B16" s="50"/>
-      <x:c r="C16" s="51"/>
-      <x:c r="D16" s="52"/>
-      <x:c r="E16" s="53"/>
-      <x:c r="F16" s="50"/>
-      <x:c r="G16" s="39"/>
-      <x:c r="H16" s="40"/>
-      <x:c r="I16" s="58"/>
-      <x:c r="J16" s="57"/>
+      <x:c r="A16" s="51"/>
+      <x:c r="B16" s="51"/>
+      <x:c r="C16" s="52"/>
+      <x:c r="D16" s="53"/>
+      <x:c r="E16" s="54"/>
+      <x:c r="F16" s="51"/>
+      <x:c r="G16" s="40"/>
+      <x:c r="H16" s="41"/>
+      <x:c r="I16" s="59"/>
+      <x:c r="J16" s="58"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
-      <x:c r="A17" s="31"/>
-      <x:c r="B17" s="31"/>
-      <x:c r="C17" s="32"/>
-      <x:c r="D17" s="33"/>
-      <x:c r="E17" s="34"/>
-      <x:c r="F17" s="31"/>
-      <x:c r="G17" s="39"/>
-      <x:c r="H17" s="40"/>
-      <x:c r="I17" s="41"/>
-      <x:c r="J17" s="38"/>
+      <x:c r="A17" s="32"/>
+      <x:c r="B17" s="32"/>
+      <x:c r="C17" s="33"/>
+      <x:c r="D17" s="34"/>
+      <x:c r="E17" s="35"/>
+      <x:c r="F17" s="32"/>
+      <x:c r="G17" s="40"/>
+      <x:c r="H17" s="41"/>
+      <x:c r="I17" s="42"/>
+      <x:c r="J17" s="39"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
-      <x:c r="A18" s="50"/>
-      <x:c r="B18" s="50"/>
-      <x:c r="C18" s="51"/>
-      <x:c r="D18" s="52"/>
-      <x:c r="E18" s="53"/>
-      <x:c r="F18" s="50"/>
-      <x:c r="G18" s="39"/>
-      <x:c r="H18" s="40"/>
-      <x:c r="I18" s="58"/>
-      <x:c r="J18" s="57"/>
+      <x:c r="A18" s="51"/>
+      <x:c r="B18" s="51"/>
+      <x:c r="C18" s="52"/>
+      <x:c r="D18" s="53"/>
+      <x:c r="E18" s="54"/>
+      <x:c r="F18" s="51"/>
+      <x:c r="G18" s="40"/>
+      <x:c r="H18" s="41"/>
+      <x:c r="I18" s="59"/>
+      <x:c r="J18" s="58"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
-      <x:c r="A19" s="31"/>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="32"/>
-      <x:c r="D19" s="33"/>
-      <x:c r="E19" s="34"/>
-      <x:c r="F19" s="31"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="40"/>
-      <x:c r="I19" s="41"/>
-      <x:c r="J19" s="38"/>
+      <x:c r="A19" s="32"/>
+      <x:c r="B19" s="32"/>
+      <x:c r="C19" s="33"/>
+      <x:c r="D19" s="34"/>
+      <x:c r="E19" s="35"/>
+      <x:c r="F19" s="32"/>
+      <x:c r="G19" s="40"/>
+      <x:c r="H19" s="41"/>
+      <x:c r="I19" s="42"/>
+      <x:c r="J19" s="39"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
-      <x:c r="A20" s="50"/>
-      <x:c r="B20" s="50"/>
-      <x:c r="C20" s="51"/>
-      <x:c r="D20" s="52"/>
-      <x:c r="E20" s="53"/>
-      <x:c r="F20" s="50"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="40"/>
-      <x:c r="I20" s="58"/>
-      <x:c r="J20" s="57"/>
+      <x:c r="A20" s="51"/>
+      <x:c r="B20" s="51"/>
+      <x:c r="C20" s="52"/>
+      <x:c r="D20" s="53"/>
+      <x:c r="E20" s="54"/>
+      <x:c r="F20" s="51"/>
+      <x:c r="G20" s="40"/>
+      <x:c r="H20" s="41"/>
+      <x:c r="I20" s="59"/>
+      <x:c r="J20" s="58"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
-      <x:c r="A21" s="31"/>
-      <x:c r="B21" s="31"/>
-      <x:c r="C21" s="32"/>
-      <x:c r="D21" s="33"/>
-      <x:c r="E21" s="34"/>
-      <x:c r="F21" s="31"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="40"/>
-      <x:c r="I21" s="41"/>
-      <x:c r="J21" s="38"/>
+      <x:c r="A21" s="32"/>
+      <x:c r="B21" s="32"/>
+      <x:c r="C21" s="33"/>
+      <x:c r="D21" s="34"/>
+      <x:c r="E21" s="35"/>
+      <x:c r="F21" s="32"/>
+      <x:c r="G21" s="40"/>
+      <x:c r="H21" s="41"/>
+      <x:c r="I21" s="42"/>
+      <x:c r="J21" s="39"/>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
-      <x:c r="A22" s="50"/>
-      <x:c r="B22" s="50"/>
-      <x:c r="C22" s="51"/>
-      <x:c r="D22" s="52"/>
-      <x:c r="E22" s="53"/>
-      <x:c r="F22" s="50"/>
-      <x:c r="G22" s="39"/>
-      <x:c r="H22" s="40"/>
-      <x:c r="I22" s="58"/>
-      <x:c r="J22" s="57"/>
+      <x:c r="A22" s="51"/>
+      <x:c r="B22" s="51"/>
+      <x:c r="C22" s="52"/>
+      <x:c r="D22" s="53"/>
+      <x:c r="E22" s="54"/>
+      <x:c r="F22" s="51"/>
+      <x:c r="G22" s="40"/>
+      <x:c r="H22" s="41"/>
+      <x:c r="I22" s="59"/>
+      <x:c r="J22" s="58"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
-      <x:c r="A23" s="31"/>
-      <x:c r="B23" s="31"/>
-      <x:c r="C23" s="32"/>
-      <x:c r="D23" s="33"/>
-      <x:c r="E23" s="34"/>
-      <x:c r="F23" s="31"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="40"/>
-      <x:c r="I23" s="41"/>
-      <x:c r="J23" s="38"/>
+      <x:c r="A23" s="32"/>
+      <x:c r="B23" s="32"/>
+      <x:c r="C23" s="33"/>
+      <x:c r="D23" s="34"/>
+      <x:c r="E23" s="35"/>
+      <x:c r="F23" s="32"/>
+      <x:c r="G23" s="40"/>
+      <x:c r="H23" s="41"/>
+      <x:c r="I23" s="42"/>
+      <x:c r="J23" s="39"/>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
-      <x:c r="A24" s="50"/>
-      <x:c r="B24" s="50"/>
-      <x:c r="C24" s="51"/>
-      <x:c r="D24" s="52"/>
-      <x:c r="E24" s="53"/>
-      <x:c r="F24" s="50"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="40"/>
-      <x:c r="I24" s="58"/>
-      <x:c r="J24" s="57"/>
+      <x:c r="A24" s="51"/>
+      <x:c r="B24" s="51"/>
+      <x:c r="C24" s="52"/>
+      <x:c r="D24" s="53"/>
+      <x:c r="E24" s="54"/>
+      <x:c r="F24" s="51"/>
+      <x:c r="G24" s="40"/>
+      <x:c r="H24" s="41"/>
+      <x:c r="I24" s="59"/>
+      <x:c r="J24" s="58"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="G5:G200">
@@ -962,20 +954,15 @@
       <x:formula>"已放弃"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H5:H200">
-    <x:cfRule type="expression" dxfId="6" priority="7">
-      <x:formula>AND(ISNUMBER(H5),H5&lt;=TODAY(),$G5&lt;&gt;"已录用",$G5&lt;&gt;"未通过",$G5&lt;&gt;"已放弃")</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G5:G200">
       <x:formula1>"已投递,已回复,面试中,已录用,未通过,已放弃,投递失败,发送待核实"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63612bb17a4848a1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R035b271e33e14e9f"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R682da7e077b249bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ba32dcb3ce0411d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>